<commit_message>
Primeros ajustes de colores, hay que seguir probando
</commit_message>
<xml_diff>
--- a/posts/Modulo2/tablaFrecuencias.xlsx
+++ b/posts/Modulo2/tablaFrecuencias.xlsx
@@ -11,6 +11,80 @@
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+  <si>
+    <t>idenpa</t>
+  </si>
+  <si>
+    <t>democ</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>frecRela</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Uruguay</t>
+  </si>
+  <si>
+    <t>Acuerdo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Argentina</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chile</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> El Salvador</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Brasil</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Costa Rica</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rep. Dominicana</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Colombia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bolivia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Venezuela</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Paraguay</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Honduras</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Peru</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Guatemala</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Panama</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ecuador</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -354,43 +428,29 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>idenpa</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>democ</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>frecRela</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Uruguay</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
       </c>
       <c r="C2">
         <v>1019</v>
@@ -402,16 +462,12 @@
         <v>0.8491666666666666</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Argentina</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
       </c>
       <c r="C3">
         <v>974</v>
@@ -423,16 +479,12 @@
         <v>0.8116666666666666</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Chile</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
       </c>
       <c r="C4">
         <v>969</v>
@@ -444,16 +496,12 @@
         <v>0.8075</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> El Salvador</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
       </c>
       <c r="C5">
         <v>803</v>
@@ -465,16 +513,12 @@
         <v>0.803</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Brasil</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
       </c>
       <c r="C6">
         <v>909</v>
@@ -486,16 +530,12 @@
         <v>0.7549833887043189</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Costa Rica</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
       </c>
       <c r="C7">
         <v>722</v>
@@ -507,16 +547,12 @@
         <v>0.722</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Mexico</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
       </c>
       <c r="C8">
         <v>857</v>
@@ -528,16 +564,12 @@
         <v>0.7141666666666666</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Rep. Dominicana</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
       </c>
       <c r="C9">
         <v>677</v>
@@ -549,16 +581,12 @@
         <v>0.677</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Colombia</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
       </c>
       <c r="C10">
         <v>757</v>
@@ -570,16 +598,12 @@
         <v>0.6308333333333334</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Bolivia</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
       </c>
       <c r="C11">
         <v>756</v>
@@ -591,16 +615,12 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Venezuela</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
       </c>
       <c r="C12">
         <v>734</v>
@@ -612,16 +632,12 @@
         <v>0.611157368859284</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Paraguay</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
       </c>
       <c r="C13">
         <v>705</v>
@@ -633,16 +649,12 @@
         <v>0.5875</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Honduras</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
       </c>
       <c r="C14">
         <v>553</v>
@@ -654,16 +666,12 @@
         <v>0.553</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Peru</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
       </c>
       <c r="C15">
         <v>649</v>
@@ -675,16 +683,12 @@
         <v>0.5408333333333334</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Guatemala</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
       </c>
       <c r="C16">
         <v>521</v>
@@ -696,16 +700,12 @@
         <v>0.521</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Panama</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
       </c>
       <c r="C17">
         <v>501</v>
@@ -717,16 +717,12 @@
         <v>0.501</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Ecuador</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Acuerdo</t>
-        </is>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
       </c>
       <c r="C18">
         <v>593</v>

</xml_diff>